<commit_message>
docs(planilhas): atualiza gestao financeira
</commit_message>
<xml_diff>
--- a/Planilhas/gestao_financeira_ouvidoria.xlsx
+++ b/Planilhas/gestao_financeira_ouvidoria.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://justicagovbr-my.sharepoint.com/personal/marcelo_cortez_mj_gov_br1/Documents/1. SENAPPEN/2. OUVIDORIA/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://justicagovbr-my.sharepoint.com/personal/marcelo_cortez_mj_gov_br1/Documents/1. SENAPPEN/2. OUVIDORIA/GITHUB/FOMENTO-ONASP/FOMENTO-ONASP/Planilhas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2130" documentId="121_{5868839F-5262-4ADE-9247-AEFBBF16C63D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{211B54AB-72F0-4619-9BE0-02DF097A9E4E}"/>
+  <xr:revisionPtr revIDLastSave="2131" documentId="121_{5868839F-5262-4ADE-9247-AEFBBF16C63D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7AA0E43D-A04F-4F72-8D5B-DF44E828614B}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{44B50A01-45D3-4E57-8B52-1C8142123E50}"/>
   </bookViews>
@@ -3306,11 +3306,11 @@
   <dxfs count="51">
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
+        <color rgb="FF006100"/>
       </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3326,11 +3326,11 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF006100"/>
+        <color rgb="FF9C0006"/>
       </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3386,21 +3386,21 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color theme="7" tint="-0.499984740745262"/>
       </font>
       <fill>
         <patternFill>
           <bgColor theme="7" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3416,11 +3416,11 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF006100"/>
+        <color rgb="FF9C0006"/>
       </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3436,11 +3436,11 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
+        <color rgb="FF006100"/>
       </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3646,6 +3646,16 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -3666,26 +3676,6 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
         <color rgb="FF9C5700"/>
       </font>
       <fill>
@@ -3701,6 +3691,16 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3830,10 +3830,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4298,8 +4294,8 @@
         <v>36509.71</v>
       </c>
       <c r="R2" s="51">
-        <f>IFERROR(SUMIFS(MT!$K:$K, MT!$A:$A, $A2, MT!$C:$C, $C2), 0)</f>
-        <v>337453.87</v>
+        <f>N3</f>
+        <v>26067.41</v>
       </c>
       <c r="S2" s="51">
         <f>IFERROR(SUMIFS(MT!$J:$J, MT!$E:$E, "OUVIDORIA", MT!$A:$A, $A2, MT!$C:$C, $C2), 0)</f>
@@ -20482,26 +20478,26 @@
     <mergeCell ref="H1:M1"/>
   </mergeCells>
   <conditionalFormatting sqref="H3:H22">
-    <cfRule type="cellIs" dxfId="39" priority="436" operator="lessThan">
+    <cfRule type="cellIs" dxfId="39" priority="438" operator="greaterThan">
+      <formula>0.7</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="38" priority="436" operator="lessThan">
       <formula>0.1</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="38" priority="437" operator="between">
+    <cfRule type="cellIs" dxfId="37" priority="437" operator="between">
       <formula>0.1</formula>
-      <formula>0.7</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="37" priority="438" operator="greaterThan">
       <formula>0.7</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I3:I22">
-    <cfRule type="containsText" dxfId="36" priority="328" operator="containsText" text="APENAS BENS">
-      <formula>NOT(ISERROR(SEARCH("APENAS BENS",I3)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="35" priority="329" operator="containsText" text="MAJORITARIAMENTE BENS">
+    <cfRule type="containsText" dxfId="36" priority="329" operator="containsText" text="MAJORITARIAMENTE BENS">
       <formula>NOT(ISERROR(SEARCH("MAJORITARIAMENTE BENS",I3)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="34" priority="330" operator="containsText" text="SERVIÇOS">
+    <cfRule type="containsText" dxfId="35" priority="330" operator="containsText" text="SERVIÇOS">
       <formula>NOT(ISERROR(SEARCH("SERVIÇOS",I3)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="34" priority="328" operator="containsText" text="APENAS BENS">
+      <formula>NOT(ISERROR(SEARCH("APENAS BENS",I3)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J3:J22">
@@ -20592,15 +20588,15 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P3:P22">
-    <cfRule type="cellIs" dxfId="13" priority="402" operator="lessThan">
-      <formula>0.1</formula>
+    <cfRule type="cellIs" dxfId="13" priority="404" operator="greaterThan">
+      <formula>0.7</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="12" priority="403" operator="between">
       <formula>0.1</formula>
       <formula>0.7</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="11" priority="404" operator="greaterThan">
-      <formula>0.7</formula>
+    <cfRule type="cellIs" dxfId="11" priority="402" operator="lessThan">
+      <formula>0.1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q3:Q5">
@@ -20609,11 +20605,11 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q3:Q22">
-    <cfRule type="containsText" dxfId="9" priority="1" operator="containsText" text="APENAS BENS">
+    <cfRule type="containsText" dxfId="9" priority="2" operator="containsText" text="MAJORITARIAMENTE BENS">
+      <formula>NOT(ISERROR(SEARCH("MAJORITARIAMENTE BENS",Q3)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="8" priority="1" operator="containsText" text="APENAS BENS">
       <formula>NOT(ISERROR(SEARCH("APENAS BENS",Q3)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="8" priority="2" operator="containsText" text="MAJORITARIAMENTE BENS">
-      <formula>NOT(ISERROR(SEARCH("MAJORITARIAMENTE BENS",Q3)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q6">
@@ -20639,14 +20635,14 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S3:S22">
-    <cfRule type="containsText" dxfId="2" priority="14" operator="containsText" text="APENAS BENS">
-      <formula>NOT(ISERROR(SEARCH("APENAS BENS",S3)))</formula>
+    <cfRule type="containsText" dxfId="2" priority="16" operator="containsText" text="SERVIÇOS">
+      <formula>NOT(ISERROR(SEARCH("SERVIÇOS",S3)))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="1" priority="15" operator="containsText" text="MAJORITARIAMENTE BENS">
       <formula>NOT(ISERROR(SEARCH("MAJORITARIAMENTE BENS",S3)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="0" priority="16" operator="containsText" text="SERVIÇOS">
-      <formula>NOT(ISERROR(SEARCH("SERVIÇOS",S3)))</formula>
+    <cfRule type="containsText" dxfId="0" priority="14" operator="containsText" text="APENAS BENS">
+      <formula>NOT(ISERROR(SEARCH("APENAS BENS",S3)))</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>

</xml_diff>

<commit_message>
Atualiza dados do relatório PROFOR 2022 e ajusta valores no JSON de publicação, incluindo correções em saldos e datas de geração. Remove itens desnecessários e ajusta totais para refletir as mudanças nos dados processados.
</commit_message>
<xml_diff>
--- a/Planilhas/gestao_financeira_ouvidoria.xlsx
+++ b/Planilhas/gestao_financeira_ouvidoria.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://justicagovbr-my.sharepoint.com/personal/marcelo_cortez_mj_gov_br1/Documents/1. SENAPPEN/2. OUVIDORIA/GITHUB/FOMENTO-ONASP/FOMENTO-ONASP/Planilhas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2170" documentId="121_{5868839F-5262-4ADE-9247-AEFBBF16C63D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E94B4A7C-8EC7-4ECB-8B75-01857993ABD8}"/>
+  <xr:revisionPtr revIDLastSave="2174" documentId="121_{5868839F-5262-4ADE-9247-AEFBBF16C63D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7CD7D9F8-2F52-40B6-B5DF-C3A5FD93407F}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="6" xr2:uid="{44B50A01-45D3-4E57-8B52-1C8142123E50}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="8" xr2:uid="{44B50A01-45D3-4E57-8B52-1C8142123E50}"/>
   </bookViews>
   <sheets>
     <sheet name="Geral" sheetId="1" r:id="rId1"/>
@@ -3282,6 +3282,9 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3295,9 +3298,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="10" fontId="6" fillId="5" borderId="25" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -18845,35 +18845,35 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:19" s="84" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="154" t="s">
+      <c r="A1" s="155" t="s">
         <v>63</v>
       </c>
-      <c r="B1" s="155"/>
-      <c r="C1" s="156"/>
+      <c r="B1" s="156"/>
+      <c r="C1" s="157"/>
       <c r="D1" s="93"/>
       <c r="E1" s="86"/>
       <c r="F1" s="86"/>
       <c r="G1" s="104"/>
-      <c r="H1" s="154" t="s">
+      <c r="H1" s="155" t="s">
         <v>64</v>
       </c>
-      <c r="I1" s="155"/>
-      <c r="J1" s="155"/>
-      <c r="K1" s="155"/>
-      <c r="L1" s="155"/>
-      <c r="M1" s="156"/>
-      <c r="N1" s="157" t="s">
+      <c r="I1" s="156"/>
+      <c r="J1" s="156"/>
+      <c r="K1" s="156"/>
+      <c r="L1" s="156"/>
+      <c r="M1" s="157"/>
+      <c r="N1" s="158" t="s">
         <v>65</v>
       </c>
-      <c r="O1" s="158"/>
-      <c r="P1" s="157" t="s">
+      <c r="O1" s="159"/>
+      <c r="P1" s="158" t="s">
         <v>66</v>
       </c>
-      <c r="Q1" s="158"/>
-      <c r="R1" s="157" t="s">
+      <c r="Q1" s="159"/>
+      <c r="R1" s="158" t="s">
         <v>67</v>
       </c>
-      <c r="S1" s="158"/>
+      <c r="S1" s="159"/>
     </row>
     <row r="2" spans="1:19" s="4" customFormat="1" ht="47.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="96" t="s">
@@ -22240,7 +22240,7 @@
       <c r="K23" s="53">
         <v>3270.64</v>
       </c>
-      <c r="L23" s="159">
+      <c r="L23" s="154">
         <f>J23-K23</f>
         <v>3950.68</v>
       </c>

</xml_diff>